<commit_message>
feat(forms): EN-26 Phase 2 Word import and EN-50 layout backlog
Add structured .docx table extractor (EN-37) with shared table parser,
wire Excel and Word through the API and FormImportPanel (EN-38), and
document EN-50 layout-heuristic Excel import with fixtures and ADR-0015.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/apps/api/test/fixtures/form-import/trade-licence-template.xlsx
+++ b/apps/api/test/fixtures/form-import/trade-licence-template.xlsx
@@ -1,41 +1,103 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\enagar\apps\api\test\fixtures\form-import\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+  </bookViews>
   <sheets>
     <sheet name="fields" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+  <si>
+    <t>field_id</t>
+  </si>
+  <si>
+    <t>label_en</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>options</t>
+  </si>
+  <si>
+    <t>business-section</t>
+  </si>
+  <si>
+    <t>Business details</t>
+  </si>
+  <si>
+    <t>section</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>trade_name</t>
+  </si>
+  <si>
+    <t>Trade name</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>trade_type</t>
+  </si>
+  <si>
+    <t>Trade type</t>
+  </si>
+  <si>
+    <t>select</t>
+  </si>
+  <si>
+    <t>retail:Retail|food:Food|services:Services</t>
+  </si>
+  <si>
+    <t>annual_turnover</t>
+  </si>
+  <si>
+    <t>Annual turnover (INR)</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>supporting-doc</t>
+  </si>
+  <si>
+    <t>Supporting document</t>
+  </si>
+  <si>
+    <t>file</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -72,6 +134,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,114 +466,122 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>field_id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>label_en</v>
-      </c>
-      <c r="C1" t="str">
-        <v>type</v>
-      </c>
-      <c r="D1" t="str">
-        <v>required</v>
-      </c>
-      <c r="E1" t="str">
-        <v>options</v>
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>business-section</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Business details</v>
-      </c>
-      <c r="C2" t="str">
-        <v>section</v>
-      </c>
-      <c r="D2" t="str">
-        <v>false</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>trade_name</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Trade name</v>
-      </c>
-      <c r="C3" t="str">
-        <v>text</v>
-      </c>
-      <c r="D3" t="str">
-        <v>true</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>trade_type</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Trade type</v>
-      </c>
-      <c r="C4" t="str">
-        <v>select</v>
-      </c>
-      <c r="D4" t="str">
-        <v>true</v>
-      </c>
-      <c r="E4" t="str">
-        <v>retail:Retail|food:Food|services:Services</v>
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>annual_turnover</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Annual turnover (INR)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>number</v>
-      </c>
-      <c r="D5" t="str">
-        <v>false</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
+    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>supporting-doc</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Supporting document</v>
-      </c>
-      <c r="C6" t="str">
-        <v>file</v>
-      </c>
-      <c r="D6" t="str">
-        <v>false</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError sqref="A1:E6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(forms): EN-26 Phase 3 PDF import (EN-39–EN-42)
Add AcroForm, digital-text, and OCR PDF extractors with EN-41 handwritten
rejection gate, PDF fixtures/runbook, and FormImportPanel .pdf support.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/apps/api/test/fixtures/form-import/trade-licence-template.xlsx
+++ b/apps/api/test/fixtures/form-import/trade-licence-template.xlsx
@@ -1,103 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\enagar\apps\api\test\fixtures\form-import\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
-  </bookViews>
   <sheets>
     <sheet name="fields" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
-  <si>
-    <t>field_id</t>
-  </si>
-  <si>
-    <t>label_en</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>options</t>
-  </si>
-  <si>
-    <t>business-section</t>
-  </si>
-  <si>
-    <t>Business details</t>
-  </si>
-  <si>
-    <t>section</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>trade_name</t>
-  </si>
-  <si>
-    <t>Trade name</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>trade_type</t>
-  </si>
-  <si>
-    <t>Trade type</t>
-  </si>
-  <si>
-    <t>select</t>
-  </si>
-  <si>
-    <t>retail:Retail|food:Food|services:Services</t>
-  </si>
-  <si>
-    <t>annual_turnover</t>
-  </si>
-  <si>
-    <t>Annual turnover (INR)</t>
-  </si>
-  <si>
-    <t>number</t>
-  </si>
-  <si>
-    <t>supporting-doc</t>
-  </si>
-  <si>
-    <t>Supporting document</t>
-  </si>
-  <si>
-    <t>file</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -134,14 +72,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -466,122 +396,114 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>field_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>label_en</v>
+      </c>
+      <c r="C1" t="str">
+        <v>type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>required</v>
+      </c>
+      <c r="E1" t="str">
+        <v>options</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>business-section</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Business details</v>
+      </c>
+      <c r="C2" t="str">
+        <v>section</v>
+      </c>
+      <c r="D2" t="str">
+        <v>false</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>trade_name</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Trade name</v>
+      </c>
+      <c r="C3" t="str">
+        <v>text</v>
+      </c>
+      <c r="D3" t="str">
+        <v>true</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>17</v>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>trade_type</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Trade type</v>
+      </c>
+      <c r="C4" t="str">
+        <v>select</v>
+      </c>
+      <c r="D4" t="str">
+        <v>true</v>
+      </c>
+      <c r="E4" t="str">
+        <v>retail:Retail|food:Food|services:Services</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>annual_turnover</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Annual turnover (INR)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>number</v>
+      </c>
+      <c r="D5" t="str">
+        <v>false</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>supporting-doc</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Supporting document</v>
+      </c>
+      <c r="C6" t="str">
+        <v>file</v>
+      </c>
+      <c r="D6" t="str">
+        <v>false</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E6" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>